<commit_message>
Update reports 2026-10-02 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-02.xlsx
+++ b/gex_pivot_levels_2026-10-02.xlsx
@@ -668,12 +668,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$10.92M</t>
+          <t>-$9.61M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$14.57M</t>
+          <t>+$12.82M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -701,12 +701,12 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-$1.97M</t>
+          <t>-$1.75M</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>+$2.98M</t>
+          <t>+$2.65M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -734,12 +734,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-$17.53M</t>
+          <t>-$16.21M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$22.77M</t>
+          <t>+$20.90M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>-$7.09M</t>
+          <t>-$6.95M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$21.33M</t>
+          <t>+$20.37M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>-$2.38M</t>
+          <t>-$2.30M</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>+$28.68M</t>
+          <t>+$27.80M</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1023,12 +1023,12 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>+$9.85M</t>
+          <t>+$10.51M</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>+$31.09M</t>
+          <t>+$33.16M</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>+$2.53M</t>
+          <t>+$2.82M</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>+$7.83M</t>
+          <t>+$8.74M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1184,12 +1184,12 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>+$21.35M</t>
+          <t>+$24.16M</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>+$34.93M</t>
+          <t>+$39.53M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -4409,76 +4409,76 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="2" t="n">
+        <v>7826.3</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>+$24.16M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>+$39.53M</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
         <v>7782.99</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C16" s="5" t="n">
         <v>768</v>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>+$1.50M</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>+$37.67M</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>2846.98</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>283</v>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>-$20.71M</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>+$36.43M</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4487,28 +4487,28 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>7826.3</v>
+        <v>2846.98</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>7750</v>
+        <v>283</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>+$21.35M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>-$20.71M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>+$34.93M</t>
+          <t>+$36.43M</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -4518,7 +4518,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4561,106 +4561,102 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>7801.3</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>7725</v>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>+$10.51M</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>+$33.16M</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B20" s="2" t="n">
         <v>4175.18</v>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C20" s="2" t="n">
         <v>380</v>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>-$25.53M</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>+$32.84M</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>2806.74</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>279</v>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>-$14.75M</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>+$32.27M</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>30756.7</v>
+        <v>2806.74</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>739</v>
+        <v>279</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>-$21.81M</t>
+          <t>-$14.75M</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>+$31.93M</t>
+          <t>+$32.27M</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -4670,7 +4666,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4681,10 +4677,10 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>30592.28</v>
+        <v>30756.7</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -4693,46 +4689,50 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>-$13.55M</t>
+          <t>-$21.81M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>+$31.51M</t>
+          <t>+$31.93M</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>7801.3</v>
+        <v>30592.28</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>7725</v>
+        <v>735</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>+$9.85M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>-$13.55M</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>+$31.09M</t>
+          <t>+$31.51M</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -4799,12 +4799,12 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>-$2.38M</t>
+          <t>-$2.30M</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>+$28.68M</t>
+          <t>+$27.80M</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -4963,102 +4963,102 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>31414.39</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>755</v>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>+$20.95M</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>+$21.30M</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B31" s="2" t="n">
         <v>7701.3</v>
       </c>
-      <c r="C30" s="2" t="n">
+      <c r="C31" s="2" t="n">
         <v>7625</v>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>-$17.53M</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>+$22.77M</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>7726.3</v>
-      </c>
-      <c r="C31" s="5" t="n">
-        <v>7650</v>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>-$7.09M</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>+$21.33M</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>-$16.21M</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>+$20.90M</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>31414.39</v>
+        <v>7726.3</v>
       </c>
       <c r="C32" s="5" t="n">
-        <v>755</v>
+        <v>7650</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>+$20.95M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>-$6.95M</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>+$21.30M</t>
+          <t>+$20.37M</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -5231,12 +5231,12 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>-$10.92M</t>
+          <t>-$9.61M</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>+$14.57M</t>
+          <t>+$12.82M</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -5397,28 +5397,28 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>31085.54</v>
+        <v>7821.3</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>747</v>
+        <v>7745</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>+$4.09M</t>
+          <t>+$2.82M</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>+$8.69M</t>
+          <t>+$8.74M</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -5435,28 +5435,28 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>7821.3</v>
+        <v>31085.54</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>7745</v>
+        <v>747</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>+$2.53M</t>
+          <t>+$4.09M</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>+$7.83M</t>
+          <t>+$8.69M</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -5933,12 +5933,12 @@
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>-$1.97M</t>
+          <t>-$1.75M</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>+$2.98M</t>
+          <t>+$2.65M</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">

</xml_diff>